<commit_message>
feat(user): add quest rewards and canonical quest balance
</commit_message>
<xml_diff>
--- a/balance/source/balance-data.xlsx
+++ b/balance/source/balance-data.xlsx
@@ -2,32 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameReward" sheetId="2" r:id="R524083d57c334d82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienSpec" sheetId="4" r:id="R921585b468554f6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopProduct" sheetId="5" r:id="R07c22c5be6a6406d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GachaPool" sheetId="6" r:id="Rab5e7de633294638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienUpgradeCost" sheetId="7" r:id="R0ab39e38f98d4128"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienLevelStat" sheetId="8" r:id="Rcb79636c56a6466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpec" sheetId="9" r:id="R91edbe3ba1454da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpec" sheetId="10" r:id="Rd94c62f5b7e34c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpawn" sheetId="11" r:id="R5dd1f1cf06a94270"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldLimitBalance" sheetId="12" r:id="R733d454e8cd64c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonBalance" sheetId="13" r:id="Rf3a5e05136f24550"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MergeRule" sheetId="14" r:id="R68e491a317f243d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicChoiceBalance" sheetId="15" r:id="R665eb31f8f4e4bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonPool" sheetId="16" r:id="R6713631ba24149ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationSpec" sheetId="17" r:id="R7aa6a0a0f7c64f28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationConfig" sheetId="18" r:id="Rb6bf4df4f14141b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InjectorPool" sheetId="19" r:id="R633f30a3e3934a0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BattleReward" sheetId="20" r:id="Raa14fd40d5174b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResonanceBalance" sheetId="21" r:id="R751e52a2db764a2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlanetBattle" sheetId="22" r:id="R3d47ddddd8a4402a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingConfig" sheetId="23" r:id="R5ca46aa4be854056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingResult" sheetId="24" r:id="Rd8d28448129b493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingRecipe" sheetId="25" r:id="R7f5967ff8c5f499f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BreedingCombinationPublic" sheetId="26" r:id="Rd8701b1d83164dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyContent" sheetId="27" r:id="R5a0af78a4bc5425e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyBattleStage" sheetId="28" r:id="R201e1dc3a5cb48bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameReward" sheetId="2" r:id="R4b50614110a54873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienSpec" sheetId="4" r:id="R47828cf9304246f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopProduct" sheetId="5" r:id="Ra5941973a2f04cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GachaPool" sheetId="6" r:id="Rd3fad6474bf142a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienUpgradeCost" sheetId="7" r:id="Rebc9d6c56cec4cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienLevelStat" sheetId="8" r:id="R32902a78471744d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpec" sheetId="9" r:id="R1181bfb2e9de43af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpec" sheetId="10" r:id="R626c267e74234387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpawn" sheetId="11" r:id="R3fd16e0c0d8341b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldLimitBalance" sheetId="12" r:id="R3686aa12eaed417f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonBalance" sheetId="13" r:id="Rd3a5d06a139147b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MergeRule" sheetId="14" r:id="Read3c129ea604a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicChoiceBalance" sheetId="15" r:id="Rc8d002ccf32c4181"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonPool" sheetId="16" r:id="R4787eedaf266432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationSpec" sheetId="17" r:id="R72e742bbef7a4523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationConfig" sheetId="18" r:id="R9c8a1d6f79f24b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InjectorPool" sheetId="19" r:id="Rb78a6333ca4e4cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BattleReward" sheetId="20" r:id="Rc354b86ffb254dc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResonanceBalance" sheetId="21" r:id="R688a21ae99474f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlanetBattle" sheetId="22" r:id="R2f457fe0e51645f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingConfig" sheetId="23" r:id="R53b2b5795b05452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingResult" sheetId="24" r:id="R59704b4844f44c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingRecipe" sheetId="25" r:id="Rd2b2e6bb10214124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BreedingCombinationPublic" sheetId="26" r:id="R9c748c8d11c74266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyContent" sheetId="27" r:id="Ra85f09b86490439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyBattleStage" sheetId="28" r:id="R95624622c44b4598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest" sheetId="29" r:id="R02245a27d7c540b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuestMilestone" sheetId="30" r:id="R5bcfd622e4f34635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achievement" sheetId="32" r:id="R12d048a0b29e4cea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -169,7 +172,7 @@
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:color indexed="8"/>
@@ -210,8 +213,13 @@
       <x:color rgb="FF9C5700"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="26">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -316,6 +324,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3B5B7A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EEF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3F6382"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3F6382"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -553,7 +581,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="180">
+  <x:cellXfs count="203">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1025,6 +1053,65 @@
     <x:xf numFmtId="204" fontId="0" fillId="21" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="7" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1099,6 +1186,61 @@
     <x:tableColumn id="13" name="statusEffectType"/>
     <x:tableColumn id="14" name="statusEffectValue"/>
     <x:tableColumn id="15" name="enabled"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="QuestTable" displayName="QuestTable" ref="A1:L9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="questId"/>
+    <x:tableColumn id="2" name="cycleType"/>
+    <x:tableColumn id="3" name="title"/>
+    <x:tableColumn id="4" name="description"/>
+    <x:tableColumn id="5" name="conditionId"/>
+    <x:tableColumn id="6" name="targetAmount"/>
+    <x:tableColumn id="7" name="activityPoints"/>
+    <x:tableColumn id="8" name="rewardGold"/>
+    <x:tableColumn id="9" name="rewardUniversalPiece"/>
+    <x:tableColumn id="10" name="rewardDiamond"/>
+    <x:tableColumn id="11" name="sortOrder"/>
+    <x:tableColumn id="12" name="enabled"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="QuestMilestoneTable" displayName="QuestMilestoneTable" ref="A1:G9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="cycleType"/>
+    <x:tableColumn id="2" name="requiredActivityPoints"/>
+    <x:tableColumn id="3" name="rewardGold"/>
+    <x:tableColumn id="4" name="rewardUniversalPiece"/>
+    <x:tableColumn id="5" name="rewardDiamond"/>
+    <x:tableColumn id="6" name="sortOrder"/>
+    <x:tableColumn id="7" name="enabled"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="AchievementTable" displayName="AchievementTable" ref="A1:L28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="achievementId"/>
+    <x:tableColumn id="2" name="category"/>
+    <x:tableColumn id="3" name="tier"/>
+    <x:tableColumn id="4" name="title"/>
+    <x:tableColumn id="5" name="description"/>
+    <x:tableColumn id="6" name="conditionId"/>
+    <x:tableColumn id="7" name="targetAmount"/>
+    <x:tableColumn id="8" name="rewardGold"/>
+    <x:tableColumn id="9" name="rewardUniversalPiece"/>
+    <x:tableColumn id="10" name="rewardDiamond"/>
+    <x:tableColumn id="11" name="sortOrder"/>
+    <x:tableColumn id="12" name="enabled"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -3262,7 +3404,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R026368c862d943ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516beda01f5847d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19945,7 +20087,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b50efcd961e48c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b51d04783041ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22371,7 +22513,1703 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2913a4004ab04699"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76d2012f29f549cc"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="187" t="str">
+        <x:v>questId</x:v>
+      </x:c>
+      <x:c r="B1" s="187" t="str">
+        <x:v>cycleType</x:v>
+      </x:c>
+      <x:c r="C1" s="187" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="D1" s="187" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="E1" s="187" t="str">
+        <x:v>conditionId</x:v>
+      </x:c>
+      <x:c r="F1" s="187" t="str">
+        <x:v>targetAmount</x:v>
+      </x:c>
+      <x:c r="G1" s="187" t="str">
+        <x:v>activityPoints</x:v>
+      </x:c>
+      <x:c r="H1" s="187" t="str">
+        <x:v>rewardGold</x:v>
+      </x:c>
+      <x:c r="I1" s="187" t="str">
+        <x:v>rewardUniversalPiece</x:v>
+      </x:c>
+      <x:c r="J1" s="187" t="str">
+        <x:v>rewardDiamond</x:v>
+      </x:c>
+      <x:c r="K1" s="187" t="str">
+        <x:v>sortOrder</x:v>
+      </x:c>
+      <x:c r="L1" s="187" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="182" t="str">
+        <x:v>DAILY_PLAY_1</x:v>
+      </x:c>
+      <x:c r="B2" s="182" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C2" s="182" t="str">
+        <x:v>전투 참가</x:v>
+      </x:c>
+      <x:c r="D2" s="182" t="str">
+        <x:v>일반 협동 전투에 1회 참가</x:v>
+      </x:c>
+      <x:c r="E2" s="182" t="str">
+        <x:v>BATTLE_MATCH_PARTICIPATION</x:v>
+      </x:c>
+      <x:c r="F2" s="190" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="190" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H2" s="190" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="I2" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="190" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L2" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="188" t="str">
+        <x:v>DAILY_WAVE_20</x:v>
+      </x:c>
+      <x:c r="B3" s="188" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C3" s="188" t="str">
+        <x:v>Wave 돌파</x:v>
+      </x:c>
+      <x:c r="D3" s="188" t="str">
+        <x:v>누적 Wave 20회 클리어</x:v>
+      </x:c>
+      <x:c r="E3" s="188" t="str">
+        <x:v>BATTLE_WAVE_CLEARED</x:v>
+      </x:c>
+      <x:c r="F3" s="191" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G3" s="191" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H3" s="191" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I3" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J3" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="191" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L3" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="182" t="str">
+        <x:v>DAILY_KILL_100</x:v>
+      </x:c>
+      <x:c r="B4" s="182" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C4" s="182" t="str">
+        <x:v>Monster 처치</x:v>
+      </x:c>
+      <x:c r="D4" s="182" t="str">
+        <x:v>Monster 100마리 처치</x:v>
+      </x:c>
+      <x:c r="E4" s="182" t="str">
+        <x:v>BATTLE_MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="F4" s="190" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="G4" s="190" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H4" s="190" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I4" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J4" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="190" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L4" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="188" t="str">
+        <x:v>DAILY_WIN_1</x:v>
+      </x:c>
+      <x:c r="B5" s="188" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C5" s="188" t="str">
+        <x:v>협동 승리</x:v>
+      </x:c>
+      <x:c r="D5" s="188" t="str">
+        <x:v>일반 협동 전투에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="E5" s="188" t="str">
+        <x:v>BATTLE_MATCH_VICTORY</x:v>
+      </x:c>
+      <x:c r="F5" s="191" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="191" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H5" s="191" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="I5" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="191" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L5" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="182" t="str">
+        <x:v>WEEKLY_PLAY_10</x:v>
+      </x:c>
+      <x:c r="B6" s="182" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="C6" s="182" t="str">
+        <x:v>전투 참가</x:v>
+      </x:c>
+      <x:c r="D6" s="182" t="str">
+        <x:v>일반 협동 전투에 10회 참가</x:v>
+      </x:c>
+      <x:c r="E6" s="182" t="str">
+        <x:v>BATTLE_MATCH_PARTICIPATION</x:v>
+      </x:c>
+      <x:c r="F6" s="190" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G6" s="190" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H6" s="190" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I6" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="190" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L6" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="188" t="str">
+        <x:v>WEEKLY_WAVE_400</x:v>
+      </x:c>
+      <x:c r="B7" s="188" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="C7" s="188" t="str">
+        <x:v>Wave 돌파</x:v>
+      </x:c>
+      <x:c r="D7" s="188" t="str">
+        <x:v>누적 Wave 400회 클리어</x:v>
+      </x:c>
+      <x:c r="E7" s="188" t="str">
+        <x:v>BATTLE_WAVE_CLEARED</x:v>
+      </x:c>
+      <x:c r="F7" s="191" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="G7" s="191" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H7" s="191" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="I7" s="191" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J7" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="191" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L7" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="182" t="str">
+        <x:v>WEEKLY_KILL_1000</x:v>
+      </x:c>
+      <x:c r="B8" s="182" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="C8" s="182" t="str">
+        <x:v>Monster 처치</x:v>
+      </x:c>
+      <x:c r="D8" s="182" t="str">
+        <x:v>Monster 1,000마리 처치</x:v>
+      </x:c>
+      <x:c r="E8" s="182" t="str">
+        <x:v>BATTLE_MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="F8" s="190" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="G8" s="190" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H8" s="190" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="I8" s="190" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J8" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="190" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L8" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="188" t="str">
+        <x:v>WEEKLY_WIN_5</x:v>
+      </x:c>
+      <x:c r="B9" s="188" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="C9" s="188" t="str">
+        <x:v>협동 승리</x:v>
+      </x:c>
+      <x:c r="D9" s="188" t="str">
+        <x:v>일반 협동 전투에서 5회 승리</x:v>
+      </x:c>
+      <x:c r="E9" s="188" t="str">
+        <x:v>BATTLE_MATCH_VICTORY</x:v>
+      </x:c>
+      <x:c r="F9" s="191" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G9" s="191" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H9" s="191" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="I9" s="191" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J9" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="191" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L9" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="B2:B9">
+      <x:formula1>"DAILY,WEEKLY"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfabfb7fa6b4b4564"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="187" t="str">
+        <x:v>cycleType</x:v>
+      </x:c>
+      <x:c r="B1" s="187" t="str">
+        <x:v>requiredActivityPoints</x:v>
+      </x:c>
+      <x:c r="C1" s="187" t="str">
+        <x:v>rewardGold</x:v>
+      </x:c>
+      <x:c r="D1" s="187" t="str">
+        <x:v>rewardUniversalPiece</x:v>
+      </x:c>
+      <x:c r="E1" s="187" t="str">
+        <x:v>rewardDiamond</x:v>
+      </x:c>
+      <x:c r="F1" s="187" t="str">
+        <x:v>sortOrder</x:v>
+      </x:c>
+      <x:c r="G1" s="187" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="182" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="B2" s="190" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C2" s="190" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="D2" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="190" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="188" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="B3" s="191" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C3" s="191" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="D3" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" s="191" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G3" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="182" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="B4" s="190" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C4" s="190" t="n">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="D4" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="190" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G4" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="188" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="B5" s="191" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C5" s="191" t="n">
+        <x:v>1250</x:v>
+      </x:c>
+      <x:c r="D5" s="191" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E5" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="191" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G5" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="182" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="B6" s="190" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C6" s="190" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D6" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="190" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="188" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="B7" s="191" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C7" s="191" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D7" s="191" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E7" s="191" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="191" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G7" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="182" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="B8" s="190" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C8" s="190" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="D8" s="190" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E8" s="190" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="190" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="183" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="188" t="str">
+        <x:v>WEEKLY</x:v>
+      </x:c>
+      <x:c r="B9" s="191" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C9" s="191" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="D9" s="191" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E9" s="191" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="F9" s="191" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G9" s="189" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="A2:A9">
+      <x:formula1>"DAILY,WEEKLY"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae3cf6d05ac04424"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="21.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="23.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="9.380000114440918" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="18.75" customHeight="1">
+      <x:c r="A1" s="202" t="str">
+        <x:v>achievementId</x:v>
+      </x:c>
+      <x:c r="B1" s="202" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="C1" s="202" t="str">
+        <x:v>tier</x:v>
+      </x:c>
+      <x:c r="D1" s="202" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="E1" s="202" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="F1" s="202" t="str">
+        <x:v>conditionId</x:v>
+      </x:c>
+      <x:c r="G1" s="202" t="str">
+        <x:v>targetAmount</x:v>
+      </x:c>
+      <x:c r="H1" s="202" t="str">
+        <x:v>rewardGold</x:v>
+      </x:c>
+      <x:c r="I1" s="202" t="str">
+        <x:v>rewardUniversalPiece</x:v>
+      </x:c>
+      <x:c r="J1" s="202" t="str">
+        <x:v>rewardDiamond</x:v>
+      </x:c>
+      <x:c r="K1" s="202" t="str">
+        <x:v>sortOrder</x:v>
+      </x:c>
+      <x:c r="L1" s="202" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="18.75" customHeight="1">
+      <x:c r="A2" s="143" t="str">
+        <x:v>ACH_BATTLE_001</x:v>
+      </x:c>
+      <x:c r="B2" s="143" t="str">
+        <x:v>BATTLE</x:v>
+      </x:c>
+      <x:c r="C2" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="143" t="str">
+        <x:v>첫 방위 작전</x:v>
+      </x:c>
+      <x:c r="E2" s="143" t="str">
+        <x:v>일반 협동 전투에 1회 참가</x:v>
+      </x:c>
+      <x:c r="F2" s="143" t="str">
+        <x:v>BATTLE_MATCH_PARTICIPATION</x:v>
+      </x:c>
+      <x:c r="G2" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H2" s="198" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="I2" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L2" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="18.75" customHeight="1">
+      <x:c r="A3" s="143" t="str">
+        <x:v>ACH_BATTLE_010</x:v>
+      </x:c>
+      <x:c r="B3" s="143" t="str">
+        <x:v>BATTLE</x:v>
+      </x:c>
+      <x:c r="C3" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D3" s="143" t="str">
+        <x:v>숙련된 방위대</x:v>
+      </x:c>
+      <x:c r="E3" s="143" t="str">
+        <x:v>일반 협동 전투에 10회 참가</x:v>
+      </x:c>
+      <x:c r="F3" s="143" t="str">
+        <x:v>BATTLE_MATCH_PARTICIPATION</x:v>
+      </x:c>
+      <x:c r="G3" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H3" s="198" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I3" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J3" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="198" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L3" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="18.75" customHeight="1">
+      <x:c r="A4" s="143" t="str">
+        <x:v>ACH_BATTLE_100</x:v>
+      </x:c>
+      <x:c r="B4" s="143" t="str">
+        <x:v>BATTLE</x:v>
+      </x:c>
+      <x:c r="C4" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D4" s="143" t="str">
+        <x:v>은하의 베테랑</x:v>
+      </x:c>
+      <x:c r="E4" s="143" t="str">
+        <x:v>일반 협동 전투에 100회 참가</x:v>
+      </x:c>
+      <x:c r="F4" s="143" t="str">
+        <x:v>BATTLE_MATCH_PARTICIPATION</x:v>
+      </x:c>
+      <x:c r="G4" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H4" s="198" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="I4" s="198" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J4" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K4" s="198" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L4" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="18.75" customHeight="1">
+      <x:c r="A5" s="143" t="str">
+        <x:v>ACH_WIN_001</x:v>
+      </x:c>
+      <x:c r="B5" s="143" t="str">
+        <x:v>VICTORY</x:v>
+      </x:c>
+      <x:c r="C5" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="143" t="str">
+        <x:v>첫 승리</x:v>
+      </x:c>
+      <x:c r="E5" s="143" t="str">
+        <x:v>일반 협동 전투에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F5" s="143" t="str">
+        <x:v>BATTLE_MATCH_VICTORY</x:v>
+      </x:c>
+      <x:c r="G5" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="198" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="I5" s="198" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J5" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L5" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="18.75" customHeight="1">
+      <x:c r="A6" s="143" t="str">
+        <x:v>ACH_WIN_010</x:v>
+      </x:c>
+      <x:c r="B6" s="143" t="str">
+        <x:v>VICTORY</x:v>
+      </x:c>
+      <x:c r="C6" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" s="143" t="str">
+        <x:v>승리의 궤도</x:v>
+      </x:c>
+      <x:c r="E6" s="143" t="str">
+        <x:v>일반 협동 전투에서 10회 승리</x:v>
+      </x:c>
+      <x:c r="F6" s="143" t="str">
+        <x:v>BATTLE_MATCH_VICTORY</x:v>
+      </x:c>
+      <x:c r="G6" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H6" s="198" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="I6" s="198" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J6" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K6" s="198" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="L6" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="18.75" customHeight="1">
+      <x:c r="A7" s="143" t="str">
+        <x:v>ACH_WIN_050</x:v>
+      </x:c>
+      <x:c r="B7" s="143" t="str">
+        <x:v>VICTORY</x:v>
+      </x:c>
+      <x:c r="C7" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D7" s="143" t="str">
+        <x:v>불패의 납치단</x:v>
+      </x:c>
+      <x:c r="E7" s="143" t="str">
+        <x:v>일반 협동 전투에서 50회 승리</x:v>
+      </x:c>
+      <x:c r="F7" s="143" t="str">
+        <x:v>BATTLE_MATCH_VICTORY</x:v>
+      </x:c>
+      <x:c r="G7" s="198" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H7" s="198" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="I7" s="198" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J7" s="198" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="K7" s="198" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="L7" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="18.75" customHeight="1">
+      <x:c r="A8" s="143" t="str">
+        <x:v>ACH_WAVE_0080</x:v>
+      </x:c>
+      <x:c r="B8" s="143" t="str">
+        <x:v>WAVE</x:v>
+      </x:c>
+      <x:c r="C8" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D8" s="143" t="str">
+        <x:v>Wave 개척자</x:v>
+      </x:c>
+      <x:c r="E8" s="143" t="str">
+        <x:v>누적 Wave 80회 클리어</x:v>
+      </x:c>
+      <x:c r="F8" s="143" t="str">
+        <x:v>BATTLE_WAVE_CLEARED</x:v>
+      </x:c>
+      <x:c r="G8" s="198" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="H8" s="198" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I8" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J8" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="198" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L8" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="18.75" customHeight="1">
+      <x:c r="A9" s="143" t="str">
+        <x:v>ACH_WAVE_0800</x:v>
+      </x:c>
+      <x:c r="B9" s="143" t="str">
+        <x:v>WAVE</x:v>
+      </x:c>
+      <x:c r="C9" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D9" s="143" t="str">
+        <x:v>Wave 항해사</x:v>
+      </x:c>
+      <x:c r="E9" s="143" t="str">
+        <x:v>누적 Wave 800회 클리어</x:v>
+      </x:c>
+      <x:c r="F9" s="143" t="str">
+        <x:v>BATTLE_WAVE_CLEARED</x:v>
+      </x:c>
+      <x:c r="G9" s="198" t="n">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="H9" s="198" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="I9" s="198" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J9" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K9" s="198" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L9" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="18.75" customHeight="1">
+      <x:c r="A10" s="143" t="str">
+        <x:v>ACH_WAVE_4000</x:v>
+      </x:c>
+      <x:c r="B10" s="143" t="str">
+        <x:v>WAVE</x:v>
+      </x:c>
+      <x:c r="C10" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" s="143" t="str">
+        <x:v>끝없는 방위선</x:v>
+      </x:c>
+      <x:c r="E10" s="143" t="str">
+        <x:v>누적 Wave 4,000회 클리어</x:v>
+      </x:c>
+      <x:c r="F10" s="143" t="str">
+        <x:v>BATTLE_WAVE_CLEARED</x:v>
+      </x:c>
+      <x:c r="G10" s="198" t="n">
+        <x:v>4000</x:v>
+      </x:c>
+      <x:c r="H10" s="198" t="n">
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="I10" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J10" s="198" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="K10" s="198" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L10" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="18.75" customHeight="1">
+      <x:c r="A11" s="143" t="str">
+        <x:v>ACH_KILL_0100</x:v>
+      </x:c>
+      <x:c r="B11" s="143" t="str">
+        <x:v>MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="C11" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D11" s="143" t="str">
+        <x:v>Monster 사냥꾼</x:v>
+      </x:c>
+      <x:c r="E11" s="143" t="str">
+        <x:v>Monster 100마리 처치</x:v>
+      </x:c>
+      <x:c r="F11" s="143" t="str">
+        <x:v>BATTLE_MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="G11" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H11" s="198" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="I11" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K11" s="198" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L11" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="18.75" customHeight="1">
+      <x:c r="A12" s="143" t="str">
+        <x:v>ACH_KILL_1000</x:v>
+      </x:c>
+      <x:c r="B12" s="143" t="str">
+        <x:v>MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="C12" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D12" s="143" t="str">
+        <x:v>Monster 청소부</x:v>
+      </x:c>
+      <x:c r="E12" s="143" t="str">
+        <x:v>Monster 1,000마리 처치</x:v>
+      </x:c>
+      <x:c r="F12" s="143" t="str">
+        <x:v>BATTLE_MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="G12" s="198" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="H12" s="198" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="I12" s="198" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J12" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K12" s="198" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="L12" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="18.75" customHeight="1">
+      <x:c r="A13" s="143" t="str">
+        <x:v>ACH_KILL_10000</x:v>
+      </x:c>
+      <x:c r="B13" s="143" t="str">
+        <x:v>MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="C13" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D13" s="143" t="str">
+        <x:v>행성 포식자</x:v>
+      </x:c>
+      <x:c r="E13" s="143" t="str">
+        <x:v>Monster 10,000마리 처치</x:v>
+      </x:c>
+      <x:c r="F13" s="143" t="str">
+        <x:v>BATTLE_MONSTER_KILL</x:v>
+      </x:c>
+      <x:c r="G13" s="198" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="H13" s="198" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="I13" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J13" s="198" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="K13" s="198" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="L13" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="18.75" customHeight="1">
+      <x:c r="A14" s="143" t="str">
+        <x:v>ACH_BOSS_001</x:v>
+      </x:c>
+      <x:c r="B14" s="143" t="str">
+        <x:v>BOSS_KILL</x:v>
+      </x:c>
+      <x:c r="C14" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="143" t="str">
+        <x:v>첫 Boss 격파</x:v>
+      </x:c>
+      <x:c r="E14" s="143" t="str">
+        <x:v>Boss 1마리 처치</x:v>
+      </x:c>
+      <x:c r="F14" s="143" t="str">
+        <x:v>BATTLE_BOSS_KILL</x:v>
+      </x:c>
+      <x:c r="G14" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H14" s="198" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="I14" s="198" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J14" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K14" s="198" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="L14" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="18.75" customHeight="1">
+      <x:c r="A15" s="143" t="str">
+        <x:v>ACH_BOSS_010</x:v>
+      </x:c>
+      <x:c r="B15" s="143" t="str">
+        <x:v>BOSS_KILL</x:v>
+      </x:c>
+      <x:c r="C15" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D15" s="143" t="str">
+        <x:v>Boss 추적자</x:v>
+      </x:c>
+      <x:c r="E15" s="143" t="str">
+        <x:v>Boss 10마리 처치</x:v>
+      </x:c>
+      <x:c r="F15" s="143" t="str">
+        <x:v>BATTLE_BOSS_KILL</x:v>
+      </x:c>
+      <x:c r="G15" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H15" s="198" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="I15" s="198" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J15" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K15" s="198" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="L15" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="18.75" customHeight="1">
+      <x:c r="A16" s="143" t="str">
+        <x:v>ACH_BOSS_050</x:v>
+      </x:c>
+      <x:c r="B16" s="143" t="str">
+        <x:v>BOSS_KILL</x:v>
+      </x:c>
+      <x:c r="C16" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D16" s="143" t="str">
+        <x:v>Boss 종결자</x:v>
+      </x:c>
+      <x:c r="E16" s="143" t="str">
+        <x:v>Boss 50마리 처치</x:v>
+      </x:c>
+      <x:c r="F16" s="143" t="str">
+        <x:v>BATTLE_BOSS_KILL</x:v>
+      </x:c>
+      <x:c r="G16" s="198" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H16" s="198" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="I16" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J16" s="198" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="K16" s="198" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L16" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="18.75" customHeight="1">
+      <x:c r="A17" s="143" t="str">
+        <x:v>ACH_SUPPORT_010</x:v>
+      </x:c>
+      <x:c r="B17" s="143" t="str">
+        <x:v>SUPPORT</x:v>
+      </x:c>
+      <x:c r="C17" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="143" t="str">
+        <x:v>협동의 시작</x:v>
+      </x:c>
+      <x:c r="E17" s="143" t="str">
+        <x:v>Support Kill 10회 달성</x:v>
+      </x:c>
+      <x:c r="F17" s="143" t="str">
+        <x:v>BATTLE_SUPPORT_KILL</x:v>
+      </x:c>
+      <x:c r="G17" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H17" s="198" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="I17" s="198" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J17" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K17" s="198" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="L17" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="18.75" customHeight="1">
+      <x:c r="A18" s="143" t="str">
+        <x:v>ACH_SUPPORT_100</x:v>
+      </x:c>
+      <x:c r="B18" s="143" t="str">
+        <x:v>SUPPORT</x:v>
+      </x:c>
+      <x:c r="C18" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D18" s="143" t="str">
+        <x:v>완벽한 호흡</x:v>
+      </x:c>
+      <x:c r="E18" s="143" t="str">
+        <x:v>Support Kill 100회 달성</x:v>
+      </x:c>
+      <x:c r="F18" s="143" t="str">
+        <x:v>BATTLE_SUPPORT_KILL</x:v>
+      </x:c>
+      <x:c r="G18" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="H18" s="198" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="I18" s="198" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J18" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="K18" s="198" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="L18" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="18.75" customHeight="1">
+      <x:c r="A19" s="143" t="str">
+        <x:v>ACH_SUPPORT_1000</x:v>
+      </x:c>
+      <x:c r="B19" s="143" t="str">
+        <x:v>SUPPORT</x:v>
+      </x:c>
+      <x:c r="C19" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D19" s="143" t="str">
+        <x:v>둘이서 하나</x:v>
+      </x:c>
+      <x:c r="E19" s="143" t="str">
+        <x:v>Support Kill 1,000회 달성</x:v>
+      </x:c>
+      <x:c r="F19" s="143" t="str">
+        <x:v>BATTLE_SUPPORT_KILL</x:v>
+      </x:c>
+      <x:c r="G19" s="198" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="H19" s="198" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="I19" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J19" s="198" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="K19" s="198" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="L19" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="18.75" customHeight="1">
+      <x:c r="A20" s="143" t="str">
+        <x:v>ACH_PLANET_NEPTUNE</x:v>
+      </x:c>
+      <x:c r="B20" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C20" s="197" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="143" t="str">
+        <x:v>해왕성 수호</x:v>
+      </x:c>
+      <x:c r="E20" s="143" t="str">
+        <x:v>해왕성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F20" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:NEPTUNE</x:v>
+      </x:c>
+      <x:c r="G20" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H20" s="198" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="I20" s="198" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J20" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" s="198" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="L20" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="18.75" customHeight="1">
+      <x:c r="A21" s="143" t="str">
+        <x:v>ACH_PLANET_URANUS</x:v>
+      </x:c>
+      <x:c r="B21" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C21" s="197" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D21" s="143" t="str">
+        <x:v>천왕성 수호</x:v>
+      </x:c>
+      <x:c r="E21" s="143" t="str">
+        <x:v>천왕성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F21" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:URANUS</x:v>
+      </x:c>
+      <x:c r="G21" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H21" s="198" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="I21" s="198" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J21" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K21" s="198" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="L21" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="18.75" customHeight="1">
+      <x:c r="A22" s="143" t="str">
+        <x:v>ACH_PLANET_SATURN</x:v>
+      </x:c>
+      <x:c r="B22" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C22" s="197" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D22" s="143" t="str">
+        <x:v>토성 수호</x:v>
+      </x:c>
+      <x:c r="E22" s="143" t="str">
+        <x:v>토성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F22" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:SATURN</x:v>
+      </x:c>
+      <x:c r="G22" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H22" s="198" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="I22" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J22" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K22" s="198" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="L22" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="18.75" customHeight="1">
+      <x:c r="A23" s="143" t="str">
+        <x:v>ACH_PLANET_JUPITER</x:v>
+      </x:c>
+      <x:c r="B23" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C23" s="197" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D23" s="143" t="str">
+        <x:v>목성 수호</x:v>
+      </x:c>
+      <x:c r="E23" s="143" t="str">
+        <x:v>목성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F23" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:JUPITER</x:v>
+      </x:c>
+      <x:c r="G23" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H23" s="198" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="I23" s="198" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J23" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K23" s="198" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="L23" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="18.75" customHeight="1">
+      <x:c r="A24" s="143" t="str">
+        <x:v>ACH_PLANET_MARS</x:v>
+      </x:c>
+      <x:c r="B24" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C24" s="197" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D24" s="143" t="str">
+        <x:v>화성 수호</x:v>
+      </x:c>
+      <x:c r="E24" s="143" t="str">
+        <x:v>화성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F24" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:MARS</x:v>
+      </x:c>
+      <x:c r="G24" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H24" s="198" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="I24" s="198" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J24" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K24" s="198" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="L24" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="18.75" customHeight="1">
+      <x:c r="A25" s="143" t="str">
+        <x:v>ACH_PLANET_EARTH</x:v>
+      </x:c>
+      <x:c r="B25" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C25" s="197" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D25" s="143" t="str">
+        <x:v>지구 수호</x:v>
+      </x:c>
+      <x:c r="E25" s="143" t="str">
+        <x:v>지구에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F25" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:EARTH</x:v>
+      </x:c>
+      <x:c r="G25" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H25" s="198" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="I25" s="198" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J25" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K25" s="198" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="L25" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="18.75" customHeight="1">
+      <x:c r="A26" s="143" t="str">
+        <x:v>ACH_PLANET_VENUS</x:v>
+      </x:c>
+      <x:c r="B26" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C26" s="197" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D26" s="143" t="str">
+        <x:v>금성 수호</x:v>
+      </x:c>
+      <x:c r="E26" s="143" t="str">
+        <x:v>금성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F26" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:VENUS</x:v>
+      </x:c>
+      <x:c r="G26" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H26" s="198" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="I26" s="198" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J26" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K26" s="198" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="L26" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="18.75" customHeight="1">
+      <x:c r="A27" s="143" t="str">
+        <x:v>ACH_PLANET_MERCURY</x:v>
+      </x:c>
+      <x:c r="B27" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C27" s="197" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D27" s="143" t="str">
+        <x:v>수성 수호</x:v>
+      </x:c>
+      <x:c r="E27" s="143" t="str">
+        <x:v>수성에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F27" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:MERCURY</x:v>
+      </x:c>
+      <x:c r="G27" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H27" s="198" t="n">
+        <x:v>40000</x:v>
+      </x:c>
+      <x:c r="I27" s="198" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="J27" s="198" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K27" s="198" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="L27" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="18.75" customHeight="1">
+      <x:c r="A28" s="143" t="str">
+        <x:v>ACH_PLANET_SUN</x:v>
+      </x:c>
+      <x:c r="B28" s="143" t="str">
+        <x:v>PLANET</x:v>
+      </x:c>
+      <x:c r="C28" s="197" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D28" s="143" t="str">
+        <x:v>태양 정복</x:v>
+      </x:c>
+      <x:c r="E28" s="143" t="str">
+        <x:v>태양에서 1회 승리</x:v>
+      </x:c>
+      <x:c r="F28" s="143" t="str">
+        <x:v>BATTLE_PLANET_VICTORY:SUN</x:v>
+      </x:c>
+      <x:c r="G28" s="198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H28" s="198" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="I28" s="198" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="J28" s="198" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="K28" s="198" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="L28" s="145" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04de4826a2634f67"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(shop): add persistent catalog purchases and rewarded rerolls
Add shop balance data, Unity catalog UI and fixtures, server purchase limits and idempotency, and safe local runtime snapshots. Record validation results and deferred launch tasks; Battle hash expectation and human acceptance remain pending.
</commit_message>
<xml_diff>
--- a/balance/source/balance-data.xlsx
+++ b/balance/source/balance-data.xlsx
@@ -2,35 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameReward" sheetId="2" r:id="R4b50614110a54873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienSpec" sheetId="4" r:id="R47828cf9304246f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopProduct" sheetId="5" r:id="Ra5941973a2f04cf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GachaPool" sheetId="6" r:id="Rd3fad6474bf142a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienUpgradeCost" sheetId="7" r:id="Rebc9d6c56cec4cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienLevelStat" sheetId="8" r:id="R32902a78471744d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpec" sheetId="9" r:id="R1181bfb2e9de43af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpec" sheetId="10" r:id="R626c267e74234387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpawn" sheetId="11" r:id="R3fd16e0c0d8341b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldLimitBalance" sheetId="12" r:id="R3686aa12eaed417f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonBalance" sheetId="13" r:id="Rd3a5d06a139147b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MergeRule" sheetId="14" r:id="Read3c129ea604a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicChoiceBalance" sheetId="15" r:id="Rc8d002ccf32c4181"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonPool" sheetId="16" r:id="R4787eedaf266432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationSpec" sheetId="17" r:id="R72e742bbef7a4523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationConfig" sheetId="18" r:id="R9c8a1d6f79f24b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InjectorPool" sheetId="19" r:id="Rb78a6333ca4e4cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BattleReward" sheetId="20" r:id="Rc354b86ffb254dc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResonanceBalance" sheetId="21" r:id="R688a21ae99474f27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlanetBattle" sheetId="22" r:id="R2f457fe0e51645f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingConfig" sheetId="23" r:id="R53b2b5795b05452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingResult" sheetId="24" r:id="R59704b4844f44c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingRecipe" sheetId="25" r:id="Rd2b2e6bb10214124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BreedingCombinationPublic" sheetId="26" r:id="R9c748c8d11c74266"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyContent" sheetId="27" r:id="Ra85f09b86490439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyBattleStage" sheetId="28" r:id="R95624622c44b4598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest" sheetId="29" r:id="R02245a27d7c540b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuestMilestone" sheetId="30" r:id="R5bcfd622e4f34635"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achievement" sheetId="32" r:id="R12d048a0b29e4cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameReward" sheetId="2" r:id="Rb3906b3fe239456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienSpec" sheetId="4" r:id="Rda91336c0ee6448e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopProduct" sheetId="5" r:id="R749aca4c840e4d12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GachaPool" sheetId="6" r:id="R1ee140bef3024470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienUpgradeCost" sheetId="7" r:id="R04d525bc14a24582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienLevelStat" sheetId="8" r:id="Rb9c8c5aed14449b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpec" sheetId="9" r:id="Rca9b22f589104365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpec" sheetId="10" r:id="R18f36c5cd591472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpawn" sheetId="11" r:id="R595f791b211a4c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldLimitBalance" sheetId="12" r:id="R50e173543e294a8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonBalance" sheetId="13" r:id="R8fd8386b5c414266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MergeRule" sheetId="14" r:id="R8807f5a6c5b74aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicChoiceBalance" sheetId="15" r:id="R54bac4f393ee434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonPool" sheetId="16" r:id="R3290295a657340aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationSpec" sheetId="17" r:id="Rc892c8d821034808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MutationConfig" sheetId="18" r:id="R762e985bd5d84dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InjectorPool" sheetId="19" r:id="Rbdc13e5bc8b54d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BattleReward" sheetId="20" r:id="R3e3b978027cd4e14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResonanceBalance" sheetId="21" r:id="R8bf46a913ec7472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlanetBattle" sheetId="22" r:id="R5737f2cda1f24287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingConfig" sheetId="23" r:id="R2f5f5a3d22204082"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingResult" sheetId="24" r:id="R7776e22aa9db44e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicBreedingRecipe" sheetId="25" r:id="R1bd97a7e68704238"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BreedingCombinationPublic" sheetId="26" r:id="R4c0c839db4654081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyContent" sheetId="27" r:id="R6a824eeeeef24014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyBattleStage" sheetId="28" r:id="R5fbf50b69e96400e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest" sheetId="29" r:id="R1696f5f077504f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuestMilestone" sheetId="30" r:id="R66bfddfdd22a4bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Achievement" sheetId="32" r:id="R30d32a2476d64021"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopOffer" sheetId="33" r:id="Rba74c21692294f2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopPolicy" sheetId="34" r:id="R0d73f545b94d42b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,7 +174,7 @@
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:color indexed="8"/>
@@ -218,8 +220,19 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color indexed="8"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color indexed="8"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="26">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -344,6 +357,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF3F6382"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E1F2"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -581,7 +599,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="203">
+  <x:cellXfs count="207">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1112,6 +1130,16 @@
     <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3404,7 +3432,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R516beda01f5847d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37dc635c840d4b37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20087,7 +20115,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b51d04783041ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dc4f3d3807e4e95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22513,7 +22541,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76d2012f29f549cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb9b06a00034307"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22886,7 +22914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfabfb7fa6b4b4564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38de42ce5c51475f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23119,7 +23147,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae3cf6d05ac04424"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71ad09e93c984f51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24209,7 +24237,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04de4826a2634f67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc18bdd5f5a7a41fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24252,7 +24280,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>500.0</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="E2" t="n">
         <x:v>1.0</x:v>
@@ -24275,7 +24303,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>5000.0</x:v>
+        <x:v>3000</x:v>
       </x:c>
       <x:c r="E3" t="n">
         <x:v>10.0</x:v>
@@ -24285,6 +24313,564 @@
       </x:c>
       <x:c r="G3" t="b">
         <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12.5" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="8.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="21.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="5.75" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11.880000114440918" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="206" t="str">
+        <x:v>offerId</x:v>
+      </x:c>
+      <x:c r="B1" s="206" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="C1" s="206" t="str">
+        <x:v>currencyType</x:v>
+      </x:c>
+      <x:c r="D1" s="206" t="str">
+        <x:v>price</x:v>
+      </x:c>
+      <x:c r="E1" s="206" t="str">
+        <x:v>rewardType</x:v>
+      </x:c>
+      <x:c r="F1" s="206" t="str">
+        <x:v>rewardAmount</x:v>
+      </x:c>
+      <x:c r="G1" s="206" t="str">
+        <x:v>grade</x:v>
+      </x:c>
+      <x:c r="H1" s="206" t="str">
+        <x:v>gachaProductId</x:v>
+      </x:c>
+      <x:c r="I1" s="206" t="str">
+        <x:v>limitPeriod</x:v>
+      </x:c>
+      <x:c r="J1" s="206" t="str">
+        <x:v>limitCount</x:v>
+      </x:c>
+      <x:c r="K1" s="206" t="str">
+        <x:v>limitGroup</x:v>
+      </x:c>
+      <x:c r="L1" s="206" t="str">
+        <x:v>active</x:v>
+      </x:c>
+      <x:c r="M1" s="206" t="str">
+        <x:v>displayOrder</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="203" t="str">
+        <x:v>GACHA_SINGLE</x:v>
+      </x:c>
+      <x:c r="B2" s="203" t="str">
+        <x:v>GACHA</x:v>
+      </x:c>
+      <x:c r="C2" s="203" t="str">
+        <x:v>DIAMOND</x:v>
+      </x:c>
+      <x:c r="D2" s="203" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E2" s="203" t="str">
+        <x:v>GACHA</x:v>
+      </x:c>
+      <x:c r="F2" s="203" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="203" t="str"/>
+      <x:c r="H2" s="203" t="str">
+        <x:v>ALIEN_GACHA_SINGLE</x:v>
+      </x:c>
+      <x:c r="I2" s="203" t="str">
+        <x:v>NONE</x:v>
+      </x:c>
+      <x:c r="J2" s="203" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="203" t="str"/>
+      <x:c r="L2" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M2" s="203" t="n">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="203" t="str">
+        <x:v>GACHA_TEN</x:v>
+      </x:c>
+      <x:c r="B3" s="203" t="str">
+        <x:v>GACHA</x:v>
+      </x:c>
+      <x:c r="C3" s="203" t="str">
+        <x:v>DIAMOND</x:v>
+      </x:c>
+      <x:c r="D3" s="203" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="E3" s="203" t="str">
+        <x:v>GACHA</x:v>
+      </x:c>
+      <x:c r="F3" s="203" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G3" s="203" t="str"/>
+      <x:c r="H3" s="203" t="str">
+        <x:v>ALIEN_GACHA_TEN</x:v>
+      </x:c>
+      <x:c r="I3" s="203" t="str">
+        <x:v>NONE</x:v>
+      </x:c>
+      <x:c r="J3" s="203" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="203" t="str"/>
+      <x:c r="L3" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M3" s="203" t="n">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="203" t="str">
+        <x:v>GOLD_PACK</x:v>
+      </x:c>
+      <x:c r="B4" s="203" t="str">
+        <x:v>RESOURCE</x:v>
+      </x:c>
+      <x:c r="C4" s="203" t="str">
+        <x:v>DIAMOND</x:v>
+      </x:c>
+      <x:c r="D4" s="203" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="E4" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="F4" s="203" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="G4" s="203" t="str"/>
+      <x:c r="H4" s="203" t="str"/>
+      <x:c r="I4" s="203" t="str">
+        <x:v>DAY</x:v>
+      </x:c>
+      <x:c r="J4" s="203" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K4" s="203" t="str">
+        <x:v>GOLD_PACK</x:v>
+      </x:c>
+      <x:c r="L4" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M4" s="203" t="n">
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="203" t="str">
+        <x:v>DNA_PACK</x:v>
+      </x:c>
+      <x:c r="B5" s="203" t="str">
+        <x:v>RESOURCE</x:v>
+      </x:c>
+      <x:c r="C5" s="203" t="str">
+        <x:v>DIAMOND</x:v>
+      </x:c>
+      <x:c r="D5" s="203" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="E5" s="203" t="str">
+        <x:v>DNA</x:v>
+      </x:c>
+      <x:c r="F5" s="203" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G5" s="203" t="str"/>
+      <x:c r="H5" s="203" t="str"/>
+      <x:c r="I5" s="203" t="str">
+        <x:v>WEEK</x:v>
+      </x:c>
+      <x:c r="J5" s="203" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K5" s="203" t="str">
+        <x:v>DNA_PACK</x:v>
+      </x:c>
+      <x:c r="L5" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M5" s="203" t="n">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="203" t="str">
+        <x:v>CELL_PACK</x:v>
+      </x:c>
+      <x:c r="B6" s="203" t="str">
+        <x:v>RESOURCE</x:v>
+      </x:c>
+      <x:c r="C6" s="203" t="str">
+        <x:v>DIAMOND</x:v>
+      </x:c>
+      <x:c r="D6" s="203" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="E6" s="203" t="str">
+        <x:v>GROWTH_CELL</x:v>
+      </x:c>
+      <x:c r="F6" s="203" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G6" s="203" t="str"/>
+      <x:c r="H6" s="203" t="str"/>
+      <x:c r="I6" s="203" t="str">
+        <x:v>WEEK</x:v>
+      </x:c>
+      <x:c r="J6" s="203" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K6" s="203" t="str">
+        <x:v>CELL_PACK</x:v>
+      </x:c>
+      <x:c r="L6" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M6" s="203" t="n">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="203" t="str">
+        <x:v>DAILY_NORMAL</x:v>
+      </x:c>
+      <x:c r="B7" s="203" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C7" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="D7" s="203" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="E7" s="203" t="str">
+        <x:v>ALIEN_PIECE</x:v>
+      </x:c>
+      <x:c r="F7" s="203" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G7" s="203" t="str">
+        <x:v>NORMAL</x:v>
+      </x:c>
+      <x:c r="H7" s="203" t="str"/>
+      <x:c r="I7" s="203" t="str">
+        <x:v>DAY</x:v>
+      </x:c>
+      <x:c r="J7" s="203" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K7" s="203" t="str">
+        <x:v>DAILY_NORMAL</x:v>
+      </x:c>
+      <x:c r="L7" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M7" s="203" t="n">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="203" t="str">
+        <x:v>DAILY_EPIC</x:v>
+      </x:c>
+      <x:c r="B8" s="203" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C8" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="D8" s="203" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="E8" s="203" t="str">
+        <x:v>ALIEN_PIECE</x:v>
+      </x:c>
+      <x:c r="F8" s="203" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G8" s="203" t="str">
+        <x:v>EPIC</x:v>
+      </x:c>
+      <x:c r="H8" s="203" t="str"/>
+      <x:c r="I8" s="203" t="str">
+        <x:v>DAY</x:v>
+      </x:c>
+      <x:c r="J8" s="203" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K8" s="203" t="str">
+        <x:v>DAILY_EPIC</x:v>
+      </x:c>
+      <x:c r="L8" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M8" s="203" t="n">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="203" t="str">
+        <x:v>DAILY_UNIQUE</x:v>
+      </x:c>
+      <x:c r="B9" s="203" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C9" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="D9" s="203" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="E9" s="203" t="str">
+        <x:v>ALIEN_PIECE</x:v>
+      </x:c>
+      <x:c r="F9" s="203" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G9" s="203" t="str">
+        <x:v>UNIQUE</x:v>
+      </x:c>
+      <x:c r="H9" s="203" t="str"/>
+      <x:c r="I9" s="203" t="str">
+        <x:v>DAY</x:v>
+      </x:c>
+      <x:c r="J9" s="203" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K9" s="203" t="str">
+        <x:v>DAILY_UNIQUE</x:v>
+      </x:c>
+      <x:c r="L9" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M9" s="203" t="n">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="203" t="str">
+        <x:v>DAILY_LEGEND</x:v>
+      </x:c>
+      <x:c r="B10" s="203" t="str">
+        <x:v>DAILY</x:v>
+      </x:c>
+      <x:c r="C10" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="D10" s="203" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="E10" s="203" t="str">
+        <x:v>ALIEN_PIECE</x:v>
+      </x:c>
+      <x:c r="F10" s="203" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G10" s="203" t="str">
+        <x:v>LEGEND</x:v>
+      </x:c>
+      <x:c r="H10" s="203" t="str"/>
+      <x:c r="I10" s="203" t="str">
+        <x:v>DAY</x:v>
+      </x:c>
+      <x:c r="J10" s="203" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K10" s="203" t="str">
+        <x:v>DAILY_LEGEND</x:v>
+      </x:c>
+      <x:c r="L10" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M10" s="203" t="n">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="203" t="str">
+        <x:v>LUCKY_DNA</x:v>
+      </x:c>
+      <x:c r="B11" s="203" t="str">
+        <x:v>LUCKY</x:v>
+      </x:c>
+      <x:c r="C11" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="D11" s="203" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="E11" s="203" t="str">
+        <x:v>DNA</x:v>
+      </x:c>
+      <x:c r="F11" s="203" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G11" s="203" t="str"/>
+      <x:c r="H11" s="203" t="str"/>
+      <x:c r="I11" s="203" t="str">
+        <x:v>WEEK</x:v>
+      </x:c>
+      <x:c r="J11" s="203" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K11" s="203" t="str">
+        <x:v>LUCKY</x:v>
+      </x:c>
+      <x:c r="L11" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M11" s="203" t="n">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="203" t="str">
+        <x:v>LUCKY_CELL</x:v>
+      </x:c>
+      <x:c r="B12" s="203" t="str">
+        <x:v>LUCKY</x:v>
+      </x:c>
+      <x:c r="C12" s="203" t="str">
+        <x:v>GOLD</x:v>
+      </x:c>
+      <x:c r="D12" s="203" t="n">
+        <x:v>20000</x:v>
+      </x:c>
+      <x:c r="E12" s="203" t="str">
+        <x:v>GROWTH_CELL</x:v>
+      </x:c>
+      <x:c r="F12" s="203" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G12" s="203" t="str"/>
+      <x:c r="H12" s="203" t="str"/>
+      <x:c r="I12" s="203" t="str">
+        <x:v>WEEK</x:v>
+      </x:c>
+      <x:c r="J12" s="203" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K12" s="203" t="str">
+        <x:v>LUCKY</x:v>
+      </x:c>
+      <x:c r="L12" s="204" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M12" s="203" t="n">
+        <x:v>110</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19.75" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="21.3799991607666" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="206" t="str">
+        <x:v>policyId</x:v>
+      </x:c>
+      <x:c r="B1" s="206" t="str">
+        <x:v>resetZone</x:v>
+      </x:c>
+      <x:c r="C1" s="206" t="str">
+        <x:v>luckyWeight</x:v>
+      </x:c>
+      <x:c r="D1" s="206" t="str">
+        <x:v>luckyTotalWeight</x:v>
+      </x:c>
+      <x:c r="E1" s="206" t="str">
+        <x:v>dailyAdRerolls</x:v>
+      </x:c>
+      <x:c r="F1" s="206" t="str">
+        <x:v>discountOfferId</x:v>
+      </x:c>
+      <x:c r="G1" s="206" t="str">
+        <x:v>discountPrice</x:v>
+      </x:c>
+      <x:c r="H1" s="206" t="str">
+        <x:v>weeklyDiscountCount</x:v>
+      </x:c>
+      <x:c r="I1" s="206" t="str">
+        <x:v>adChallengeTtlSeconds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="203" t="str">
+        <x:v>DEFAULT</x:v>
+      </x:c>
+      <x:c r="B2" s="203" t="str">
+        <x:v>Asia/Seoul</x:v>
+      </x:c>
+      <x:c r="C2" s="203" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D2" s="203" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="E2" s="203" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F2" s="203" t="str">
+        <x:v>GACHA_TEN</x:v>
+      </x:c>
+      <x:c r="G2" s="203" t="n">
+        <x:v>2700</x:v>
+      </x:c>
+      <x:c r="H2" s="203" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I2" s="203" t="n">
+        <x:v>600</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>